<commit_message>
Text institute and country
</commit_message>
<xml_diff>
--- a/11-CollaborationList/ASU.xlsx
+++ b/11-CollaborationList/ASU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kennethlong/Library/CloudStorage/Box-Box/CubMac-Box/KL-GIT/CCAP/02-LhARA/00-Collaboration-lists/11-CollaborationList/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2153814637468/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542D5928-D4A3-7A4D-BBCF-4E7082F21216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{114D98B5-9F22-FC41-AF24-FF0A63D5AB15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="16200" windowWidth="57600" windowHeight="16200" xr2:uid="{5FAB20B0-5FD5-FD49-A8D1-27020549867D}"/>
+    <workbookView xWindow="0" yWindow="12600" windowWidth="51200" windowHeight="16200" xr2:uid="{5FAB20B0-5FD5-FD49-A8D1-27020549867D}"/>
   </bookViews>
   <sheets>
     <sheet name="UCL" sheetId="1" r:id="rId1"/>
@@ -88,9 +88,6 @@
     <t>ASU</t>
   </si>
   <si>
-    <t>Arizona State University: Tempe, Arizona, US</t>
-  </si>
-  <si>
     <t>0009-0004-0894-6295</t>
   </si>
   <si>
@@ -110,6 +107,9 @@
   </si>
   <si>
     <t>0000-0002-7876-855X</t>
+  </si>
+  <si>
+    <t>Arizona State University, Tempe, Arizona, US</t>
   </si>
 </sst>
 </file>
@@ -1095,13 +1095,13 @@
         <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -1109,31 +1109,31 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" t="s">
         <v>27</v>
-      </c>
-      <c r="F3" t="s">
-        <v>28</v>
       </c>
       <c r="G3" t="s">
         <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>